<commit_message>
docs: cập nhật khảo sát lên N=21 — evidence đạt trọn chuẩn A
Khảo sát bổ sung đủ ≥20 người ngoài nhóm, nên nhóm nay có cả hai
chuẩn evidence A và B của BTC.

Số liệu mới (mọi kết luận cũ đều giữ nguyên, phần lớn mạnh hơn):
- 90% từng phải hỏi lại bot · 86% phải tự kiểm tra lại câu trả lời
- 14/18 người kiểm tra lại bằng cách đi hỏi người thật
- 90% thấy bot không hoàn toàn đúng, chủ yếu "đúng một phần" (16/21)
- chờ TA lâu vẫn không phải nỗi đau chính (2/21 thường xuyên)
- lỗ hổng kho rộng hơn: Standup 95% hỏi / 0 mục, đề tài 67% / 0 mục

Cập nhật spec.md §1 §8 §9, canvas.md, feedback-log.md theo số mới.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Khảo-sát-chất-lượng-Discord-Bot-Level-34-Khóa-4-VIN-AI-20K-Câu-trả-lời.xlsx
+++ b/docs/Khảo-sát-chất-lượng-Discord-Bot-Level-34-Khóa-4-VIN-AI-20K-Câu-trả-lời.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/an/Documents/VIN AI/Lab5/K4-3A-E402-KKAL/docs/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/an/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87FDFCA7-1F2A-504D-A393-69EEF80EC9A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3FC8221-808B-624C-8B5B-8063A20DC100}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="25940" windowHeight="16960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="177" uniqueCount="54">
   <si>
     <t>1. Bạn đã từng hỏi Discord Bot trong Khóa 4 chưa?</t>
   </si>
@@ -164,6 +164,24 @@
   </si>
   <si>
     <t>Thành lập / ghép / đổi team, Daily Standup, GitHub / repository / quyền truy cập, Workshop / Office Hours, Mã đội / mã nhóm, Chọn / đổi / đề xuất đề tài</t>
+  </si>
+  <si>
+    <t>Thành lập / ghép / đổi team, Daily Standup, GitHub / repository / quyền truy cập, Workshop / Office Hours, Phoenix, Quy chế / nội dung bắt buộc, XP / điểm, Chọn / đổi / đề xuất đề tài, Ticket / liên hệ hỗ trợ</t>
+  </si>
+  <si>
+    <t>Có, qua thông báo Discord, Có, hỏi bạn học, Có, hỏi Mentor / Lab Coach / TA, Có, hỏi BTC / Mod</t>
+  </si>
+  <si>
+    <t>Thành lập / ghép / đổi team, Daily Standup, Mentor / Lab Coach, Workshop / Office Hours, Phoenix, Chọn / đổi / đề xuất đề tài</t>
+  </si>
+  <si>
+    <t>Daily Standup, Chọn / đổi / đề xuất đề tài</t>
+  </si>
+  <si>
+    <t>Thành lập / ghép / đổi team, Daily Standup, Mentor / Lab Coach, Workshop / Office Hours, Phoenix, Quy chế / nội dung bắt buộc, Lịch học / deadline, Chọn / đổi / đề xuất đề tài, Ticket / liên hệ hỗ trợ</t>
+  </si>
+  <si>
+    <t>Daily Standup, GitHub / repository / quyền truy cập, Mentor / Lab Coach, Workshop / Office Hours, Mã đội / mã nhóm, Chọn / đổi / đề xuất đề tài</t>
   </si>
 </sst>
 </file>
@@ -204,10 +222,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -282,7 +303,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Form_Responses" displayName="Form_Responses" ref="A1:I16">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Form_Responses" displayName="Form_Responses" ref="A1:I22">
   <tableColumns count="9">
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="1. Bạn đã từng hỏi Discord Bot trong Khóa 4 chưa?"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="2. Bạn sử dụng Bot với tần suất như thế nào?"/>
@@ -499,11 +520,10 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:I16"/>
+  <dimension ref="A1:I22"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
   <cols>
-    <col min="1" max="1" width="36.83203125" customWidth="1"/>
-    <col min="2" max="2" width="37.6640625" customWidth="1"/>
+    <col min="1" max="2" width="37.6640625" customWidth="1"/>
     <col min="3" max="3" width="33.6640625" customWidth="1"/>
     <col min="4" max="9" width="37.6640625" customWidth="1"/>
     <col min="10" max="15" width="18.83203125" customWidth="1"/>
@@ -973,6 +993,180 @@
         <v>27</v>
       </c>
     </row>
+    <row r="17" spans="1:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A17" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="D17" s="3">
+        <v>3</v>
+      </c>
+      <c r="E17" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F17" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="G17" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="H17" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="I17" s="3" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A18" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="D18" s="3">
+        <v>3</v>
+      </c>
+      <c r="E18" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F18" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="G18" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="H18" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="I18" s="3" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A19" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C19" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="D19" s="3">
+        <v>3</v>
+      </c>
+      <c r="E19" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="F19" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="G19" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="H19" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="I19" s="3" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A20" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C20" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="D20" s="3">
+        <v>3</v>
+      </c>
+      <c r="E20" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F20" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="G20" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="H20" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="I20" s="3" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A21" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C21" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="D21" s="3">
+        <v>3</v>
+      </c>
+      <c r="E21" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="F21" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="G21" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="H21" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="I21" s="3" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A22" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C22" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="D22" s="3">
+        <v>3</v>
+      </c>
+      <c r="E22" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F22" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="G22" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="H22" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="I22" s="3" t="s">
+        <v>16</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">

</xml_diff>